<commit_message>
Nouveau journal de groupe
</commit_message>
<xml_diff>
--- a/planning/Journal_planification_du_groupe.xlsx
+++ b/planning/Journal_planification_du_groupe.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilstan.sanquer\Desktop\Github\SquidTchat\planning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A13A662-9BFF-41C4-9B4D-77762DF6EDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDB86920-F53C-438B-A7B8-49C6FE70CEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
+    <workbookView xWindow="6810" yWindow="3600" windowWidth="21600" windowHeight="11295" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -412,18 +412,18 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-• 1h : Mise à jour du cahier de recette :</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Raphaël</t>
+• 1h15 : Mise à jour du cahier de recette : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Raphaël</t>
     </r>
     <r>
       <rPr>
@@ -434,7 +434,29 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-• 30 min : Optimisation du filtre des pseudos : </t>
+• 1h : Mise à jour de l'html / affichage du titre : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1h : Optimisation du filtre des pseudos : </t>
     </r>
     <r>
       <rPr>
@@ -725,63 +747,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -799,6 +764,63 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1156,371 +1178,371 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF07D86-D2F8-4F32-A268-7E13E7D471B5}">
   <dimension ref="A1:R28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-    </row>
-    <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+    </row>
+    <row r="3" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8" t="s">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="17" t="s">
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="19"/>
-      <c r="I3" s="17" t="s">
+      <c r="H3" s="25"/>
+      <c r="I3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="19"/>
-    </row>
-    <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="22"/>
-    </row>
-    <row r="5" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="22"/>
-    </row>
-    <row r="6" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="22"/>
-    </row>
-    <row r="7" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="22"/>
-    </row>
-    <row r="8" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="24"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
-      <c r="O8" s="24"/>
-      <c r="P8" s="24"/>
-      <c r="Q8" s="24"/>
-      <c r="R8" s="25"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="10">
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="25"/>
+    </row>
+    <row r="4" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="28"/>
+    </row>
+    <row r="5" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="28"/>
+    </row>
+    <row r="6" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="28"/>
+    </row>
+    <row r="7" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="28"/>
+    </row>
+    <row r="8" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="30"/>
+      <c r="Q8" s="30"/>
+      <c r="R8" s="31"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="16">
         <v>46094</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9" t="s">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="H9" s="4"/>
-      <c r="I9" s="26" t="s">
+      <c r="I9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
-      <c r="R9" s="28"/>
-    </row>
-    <row r="10" spans="1:18" ht="84" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="9"/>
+    </row>
+    <row r="10" spans="1:18" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="5"/>
       <c r="H10" s="6"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-      <c r="P10" s="30"/>
-      <c r="Q10" s="30"/>
-      <c r="R10" s="31"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="11">
+      <c r="I10" s="10"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="17">
         <v>46098</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="9" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="H11" s="4"/>
-      <c r="I11" s="26" t="s">
+      <c r="I11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="28"/>
-    </row>
-    <row r="12" spans="1:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="9"/>
+    </row>
+    <row r="12" spans="1:18" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="20"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="5"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="30"/>
-      <c r="Q12" s="30"/>
-      <c r="R12" s="31"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A13" s="10">
+      <c r="I12" s="10"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
         <v>46104</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="H13" s="4"/>
-      <c r="I13" s="26" t="s">
+      <c r="I13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J13" s="27"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="27"/>
-      <c r="M13" s="27"/>
-      <c r="N13" s="27"/>
-      <c r="O13" s="27"/>
-      <c r="P13" s="27"/>
-      <c r="Q13" s="27"/>
-      <c r="R13" s="28"/>
-    </row>
-    <row r="14" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="9"/>
+    </row>
+    <row r="14" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="5"/>
       <c r="H14" s="6"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="30"/>
-      <c r="O14" s="30"/>
-      <c r="P14" s="30"/>
-      <c r="Q14" s="30"/>
-      <c r="R14" s="31"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A15" s="10">
+      <c r="I14" s="10"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="16">
         <v>46115</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9" t="s">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="3" t="s">
         <v>8</v>
       </c>
       <c r="H15" s="4"/>
-      <c r="I15" s="26" t="s">
+      <c r="I15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-      <c r="O15" s="27"/>
-      <c r="P15" s="27"/>
-      <c r="Q15" s="27"/>
-      <c r="R15" s="28"/>
-    </row>
-    <row r="16" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="9"/>
+    </row>
+    <row r="16" spans="1:18" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="5"/>
       <c r="H16" s="6"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
-      <c r="P16" s="30"/>
-      <c r="Q16" s="30"/>
-      <c r="R16" s="31"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="I16" s="10"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="32"/>
       <c r="B17" s="32"/>
       <c r="C17" s="32"/>
@@ -1542,7 +1564,7 @@
       <c r="Q17" s="34"/>
       <c r="R17" s="35"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="32"/>
       <c r="B18" s="32"/>
       <c r="C18" s="32"/>
@@ -1562,7 +1584,7 @@
       <c r="Q18" s="37"/>
       <c r="R18" s="38"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="32"/>
       <c r="B19" s="32"/>
       <c r="C19" s="32"/>
@@ -1584,7 +1606,7 @@
       <c r="Q19" s="32"/>
       <c r="R19" s="32"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="32"/>
       <c r="B20" s="32"/>
       <c r="C20" s="32"/>
@@ -1604,7 +1626,7 @@
       <c r="Q20" s="32"/>
       <c r="R20" s="32"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="32"/>
       <c r="B21" s="32"/>
       <c r="C21" s="32"/>
@@ -1626,7 +1648,7 @@
       <c r="Q21" s="32"/>
       <c r="R21" s="32"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="32"/>
       <c r="B22" s="32"/>
       <c r="C22" s="32"/>
@@ -1646,7 +1668,7 @@
       <c r="Q22" s="32"/>
       <c r="R22" s="32"/>
     </row>
-    <row r="23" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1665,7 +1687,7 @@
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1685,7 +1707,7 @@
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1705,7 +1727,7 @@
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1725,7 +1747,7 @@
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1745,7 +1767,7 @@
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1805,4 +1827,239 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E3DBFDA92D80EA48A7EED411DA26BC07" ma:contentTypeVersion="9" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="8d7da3b0ce409c83d2d88bc67c89ad87">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61a5eff35266d42fcf39f049a9a05b65" ns3:_="">
+    <xsd:import namespace="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_activity" ma:index="12" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="13" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E5277FF-56CA-490A-8F5B-11638F046AC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A62BBD1-AF82-4CFC-85F1-43EAF693E720}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B75C78B4-7D45-4308-B84E-7AAC1168BFC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Maj, planif du groupe
</commit_message>
<xml_diff>
--- a/planning/Journal_planification_du_groupe.xlsx
+++ b/planning/Journal_planification_du_groupe.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDB86920-F53C-438B-A7B8-49C6FE70CEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2F7960-AEBF-48E1-B900-6A41779B744F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6810" yWindow="3600" windowWidth="21600" windowHeight="11295" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>Jour</t>
   </si>
@@ -556,6 +556,157 @@
         <scheme val="minor"/>
       </rPr>
       <t>Jean</t>
+    </r>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• 1h- 1h30 : Gestion du programme groupes </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wilstan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1/2h- 1h : Gestion de l'interfaces des groupes </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wilstan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1h30 : Finalisation des cahiers de recettes : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1h : Finalisation du filtre des pseudos : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Raphaël</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 2h : Début de réalisation de la présentation du projet : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jean</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1h- 1h30 : Intégration JavaScript – Messagerie privée : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wilstan, Raphaël et Jean</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+• 1/2h- 1h : Intégration des filtres de messages au groupes : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jean, Raphaël</t>
     </r>
   </si>
 </sst>
@@ -727,7 +878,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -822,11 +973,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -841,6 +995,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1177,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF07D86-D2F8-4F32-A268-7E13E7D471B5}">
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -1542,133 +1699,142 @@
       <c r="Q16" s="11"/>
       <c r="R16" s="12"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33" t="s">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17" s="32">
+        <v>46139</v>
+      </c>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="34"/>
-      <c r="N17" s="34"/>
-      <c r="O17" s="34"/>
-      <c r="P17" s="34"/>
-      <c r="Q17" s="34"/>
-      <c r="R17" s="35"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="37"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="37"/>
-      <c r="R18" s="38"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32" t="s">
+      <c r="H17" s="36"/>
+      <c r="I17" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="35"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="35"/>
+      <c r="Q17" s="35"/>
+      <c r="R17" s="36"/>
+      <c r="S17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="106.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="33"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="38"/>
+      <c r="N18" s="38"/>
+      <c r="O18" s="38"/>
+      <c r="P18" s="38"/>
+      <c r="Q18" s="38"/>
+      <c r="R18" s="39"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="33"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="32"/>
-      <c r="K20" s="32"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="32"/>
-      <c r="N20" s="32"/>
-      <c r="O20" s="32"/>
-      <c r="P20" s="32"/>
-      <c r="Q20" s="32"/>
-      <c r="R20" s="32"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32" t="s">
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+      <c r="P19" s="33"/>
+      <c r="Q19" s="33"/>
+      <c r="R19" s="33"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="33"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33"/>
+      <c r="Q20" s="33"/>
+      <c r="R20" s="33"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21" s="33"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="32"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="32"/>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="32"/>
-      <c r="Q22" s="32"/>
-      <c r="R22" s="32"/>
-    </row>
-    <row r="23" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
+      <c r="P21" s="33"/>
+      <c r="Q21" s="33"/>
+      <c r="R21" s="33"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22" s="33"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
+      <c r="P22" s="33"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+    </row>
+    <row r="23" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1687,7 +1853,7 @@
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1707,7 +1873,7 @@
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1727,7 +1893,7 @@
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1747,7 +1913,7 @@
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1767,7 +1933,7 @@
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>

</xml_diff>